<commit_message>
Issue 27 · 15 Jun 2026 · chips+gold rotation
</commit_message>
<xml_diff>
--- a/Parallax_Portfolio_Simple_2026-06-15.xlsx
+++ b/Parallax_Portfolio_Simple_2026-06-15.xlsx
@@ -436,12 +436,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>XLV</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -451,12 +451,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -466,12 +466,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>XLU</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -481,12 +481,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -496,12 +496,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ELV</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -511,12 +511,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -526,12 +526,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>NEM</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -541,12 +541,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>AEM</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -556,12 +556,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KMB</t>
+          <t>WPM</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -571,12 +571,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>KGC</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -586,12 +586,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>FNV</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -601,12 +601,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -616,12 +616,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>LMT</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -631,12 +631,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>VTIP</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="C15" t="n">

</xml_diff>